<commit_message>
Completar datos confirmados del cliente Matheu Marcos (CUIT verificado)
- Ficha del Excel con CUIT 20-31822115-5 tomado de la base del estudio
- Informe actualizado: cliente nuevo en base, diagnóstico ARCA ejecutable

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PCAGEfq7p7jhfQiJzYkBZA
</commit_message>
<xml_diff>
--- a/Estudio Contable/CLIENTES/ACT RESP. INSC/MATHEU MARCO/Analisis Integral y Abono - MATHEU MARCO.xlsx
+++ b/Estudio Contable/CLIENTES/ACT RESP. INSC/MATHEU MARCO/Analisis Integral y Abono - MATHEU MARCO.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="342">
   <si>
     <t xml:space="preserve">ANÁLISIS INTEGRAL DEL CLIENTE Y PROPUESTA DE ABONO</t>
   </si>
@@ -40,7 +40,7 @@
     <t xml:space="preserve">Cliente</t>
   </si>
   <si>
-    <t xml:space="preserve">MATHEU, MARCO</t>
+    <t xml:space="preserve">MATHEU, MARCOS</t>
   </si>
   <si>
     <t xml:space="preserve">Nombre comercial</t>
@@ -52,7 +52,7 @@
     <t xml:space="preserve">CUIT</t>
   </si>
   <si>
-    <t xml:space="preserve">A CONFIRMAR</t>
+    <t xml:space="preserve">20-31822115-5</t>
   </si>
   <si>
     <t xml:space="preserve">Condición fiscal</t>
@@ -62,6 +62,9 @@
   </si>
   <si>
     <t xml:space="preserve">Ingresos Brutos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A CONFIRMAR (sin dato en la base del estudio)</t>
   </si>
   <si>
     <t xml:space="preserve">Empleados declarados</t>
@@ -1946,7 +1949,7 @@
       <c r="B7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1963,49 +1966,49 @@
         <v>11</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C16" s="8" t="n">
         <f aca="false">COUNTIF(DIAGNOSTICO!$F$4:$F$21,"Pendiente")</f>
@@ -2014,7 +2017,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C17" s="9" t="n">
         <f aca="false">COUNTIF(DIAGNOSTICO!$F$4:$F$21,"OK")</f>
@@ -2023,7 +2026,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C18" s="10" t="n">
         <f aca="false">COUNTIF(DIAGNOSTICO!$F$4:$F$21,"Alerta")</f>
@@ -2032,7 +2035,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C19" s="11" t="n">
         <f aca="false">COUNTIF(DIAGNOSTICO!$F$4:$F$21,"Crítico")</f>
@@ -2041,12 +2044,12 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">ABONO!$I$27</f>
@@ -2055,7 +2058,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C23" s="12" t="n">
         <f aca="false">ABONO!$I$29</f>
@@ -2064,7 +2067,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C24" s="12" t="n">
         <f aca="false">ABONO!$I$31</f>
@@ -2073,7 +2076,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C25" s="12" t="n">
         <f aca="false">ABONO!$I$33</f>
@@ -2082,12 +2085,12 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
@@ -2096,7 +2099,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="13" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
@@ -2105,7 +2108,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="13" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C30" s="13"/>
       <c r="D30" s="13"/>
@@ -2114,7 +2117,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="13" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
@@ -2123,7 +2126,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
@@ -2132,12 +2135,12 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C35" s="15"/>
       <c r="D35" s="15"/>
@@ -2146,7 +2149,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
@@ -2155,7 +2158,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C37" s="17"/>
       <c r="D37" s="17"/>
@@ -2164,7 +2167,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="18" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C38" s="18"/>
       <c r="D38" s="18"/>
@@ -2173,7 +2176,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C40" s="19"/>
       <c r="D40" s="19"/>
@@ -2242,7 +2245,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -2256,7 +2259,7 @@
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="21" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B2" s="21"/>
       <c r="C2" s="21"/>
@@ -2270,34 +2273,34 @@
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G3" s="22" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H3" s="22" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I3" s="22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J3" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2305,31 +2308,31 @@
         <v>1</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H4" s="26" t="n">
         <v>0</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J4" s="25" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2337,27 +2340,27 @@
         <v>2</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E5" s="27"/>
       <c r="F5" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G5" s="24"/>
       <c r="H5" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2365,27 +2368,27 @@
         <v>3</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E6" s="27"/>
       <c r="F6" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G6" s="24"/>
       <c r="H6" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="24" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J6" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2393,27 +2396,27 @@
         <v>4</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E7" s="27"/>
       <c r="F7" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G7" s="24"/>
       <c r="H7" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I7" s="24" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J7" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2421,27 +2424,27 @@
         <v>5</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E8" s="27"/>
       <c r="F8" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G8" s="24"/>
       <c r="H8" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="24" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J8" s="24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2449,27 +2452,27 @@
         <v>6</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E9" s="27"/>
       <c r="F9" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G9" s="24"/>
       <c r="H9" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I9" s="24" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2477,27 +2480,27 @@
         <v>7</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E10" s="27"/>
       <c r="F10" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G10" s="24"/>
       <c r="H10" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J10" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2505,27 +2508,27 @@
         <v>8</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E11" s="27"/>
       <c r="F11" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G11" s="24"/>
       <c r="H11" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="24" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J11" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2533,27 +2536,27 @@
         <v>9</v>
       </c>
       <c r="B12" s="24" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E12" s="27"/>
       <c r="F12" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G12" s="24"/>
       <c r="H12" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="24" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J12" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2561,27 +2564,27 @@
         <v>10</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E13" s="27"/>
       <c r="F13" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G13" s="24"/>
       <c r="H13" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="24" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2589,27 +2592,27 @@
         <v>11</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D14" s="24" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E14" s="27"/>
       <c r="F14" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G14" s="24"/>
       <c r="H14" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J14" s="24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2617,27 +2620,27 @@
         <v>12</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E15" s="27"/>
       <c r="F15" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G15" s="24"/>
       <c r="H15" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="24" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J15" s="24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2645,27 +2648,27 @@
         <v>13</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C16" s="24" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D16" s="24" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E16" s="27"/>
       <c r="F16" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G16" s="24"/>
       <c r="H16" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J16" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2673,27 +2676,27 @@
         <v>14</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C17" s="24" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D17" s="24" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E17" s="27"/>
       <c r="F17" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G17" s="24"/>
       <c r="H17" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J17" s="24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2701,27 +2704,27 @@
         <v>15</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C18" s="24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D18" s="24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E18" s="27"/>
       <c r="F18" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G18" s="24"/>
       <c r="H18" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I18" s="24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J18" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2729,27 +2732,27 @@
         <v>16</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C19" s="24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D19" s="24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E19" s="27"/>
       <c r="F19" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G19" s="24"/>
       <c r="H19" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I19" s="24" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J19" s="24" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2757,27 +2760,27 @@
         <v>17</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C20" s="24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D20" s="24" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E20" s="27"/>
       <c r="F20" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G20" s="24"/>
       <c r="H20" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I20" s="24" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J20" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2785,32 +2788,32 @@
         <v>18</v>
       </c>
       <c r="B21" s="24" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C21" s="24" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D21" s="24" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E21" s="27"/>
       <c r="F21" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G21" s="24"/>
       <c r="H21" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J21" s="24" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G22" s="29" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H22" s="30" t="n">
         <f aca="false">SUM(H4:H21)</f>
@@ -2872,7 +2875,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -2883,7 +2886,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="21" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B2" s="21"/>
       <c r="C2" s="21"/>
@@ -2894,25 +2897,25 @@
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G3" s="22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2920,20 +2923,20 @@
         <v>1</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E4" s="27"/>
       <c r="F4" s="24" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2941,20 +2944,20 @@
         <v>2</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E5" s="27"/>
       <c r="F5" s="24" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2962,20 +2965,20 @@
         <v>3</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E6" s="27"/>
       <c r="F6" s="24" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2983,20 +2986,20 @@
         <v>4</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E7" s="27"/>
       <c r="F7" s="24" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3004,20 +3007,20 @@
         <v>5</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E8" s="27"/>
       <c r="F8" s="24" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3025,20 +3028,20 @@
         <v>6</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E9" s="27"/>
       <c r="F9" s="24" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3046,20 +3049,20 @@
         <v>7</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E10" s="27"/>
       <c r="F10" s="24" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3067,20 +3070,20 @@
         <v>8</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E11" s="27"/>
       <c r="F11" s="24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3088,20 +3091,20 @@
         <v>9</v>
       </c>
       <c r="B12" s="24" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E12" s="27"/>
       <c r="F12" s="24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3109,20 +3112,20 @@
         <v>10</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E13" s="27"/>
       <c r="F13" s="24" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3130,20 +3133,20 @@
         <v>11</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D14" s="24" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E14" s="27"/>
       <c r="F14" s="24" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3151,20 +3154,20 @@
         <v>12</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E15" s="27"/>
       <c r="F15" s="24" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3219,7 +3222,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -3233,34 +3236,34 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="14" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="31" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C4" s="32" t="n">
         <v>15000</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="31" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C5" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="31" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C6" s="32" t="n">
         <v>35000</v>
@@ -3268,7 +3271,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="31" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C7" s="35" t="n">
         <v>0.21</v>
@@ -3276,34 +3279,34 @@
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G8" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I8" s="22" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3311,13 +3314,13 @@
         <v>1</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D9" s="36" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E9" s="37" t="n">
         <v>3</v>
@@ -3344,13 +3347,13 @@
         <v>2</v>
       </c>
       <c r="B10" s="31" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E10" s="37" t="n">
         <v>2</v>
@@ -3377,13 +3380,13 @@
         <v>3</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D11" s="36" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E11" s="37" t="n">
         <v>2</v>
@@ -3410,13 +3413,13 @@
         <v>4</v>
       </c>
       <c r="B12" s="31" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E12" s="37" t="n">
         <v>0.5</v>
@@ -3443,13 +3446,13 @@
         <v>5</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D13" s="36" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E13" s="37" t="n">
         <v>1</v>
@@ -3476,13 +3479,13 @@
         <v>6</v>
       </c>
       <c r="B14" s="31" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E14" s="31" t="n">
         <f aca="false">1*$C$5</f>
@@ -3511,13 +3514,13 @@
         <v>7</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D15" s="36" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E15" s="37" t="n">
         <v>2</v>
@@ -3544,13 +3547,13 @@
         <v>8</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D16" s="36" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E16" s="37" t="n">
         <v>3</v>
@@ -3577,13 +3580,13 @@
         <v>9</v>
       </c>
       <c r="B17" s="31" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D17" s="36" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E17" s="37" t="n">
         <v>4</v>
@@ -3610,13 +3613,13 @@
         <v>10</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C18" s="31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D18" s="36" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E18" s="37" t="n">
         <v>2</v>
@@ -3643,13 +3646,13 @@
         <v>11</v>
       </c>
       <c r="B19" s="31" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C19" s="31" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D19" s="36" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E19" s="37" t="n">
         <v>1</v>
@@ -3676,13 +3679,13 @@
         <v>12</v>
       </c>
       <c r="B20" s="31" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C20" s="31" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E20" s="37" t="n">
         <v>0.5</v>
@@ -3709,13 +3712,13 @@
         <v>13</v>
       </c>
       <c r="B21" s="31" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C21" s="31" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D21" s="36" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E21" s="37" t="n">
         <v>1</v>
@@ -3742,13 +3745,13 @@
         <v>14</v>
       </c>
       <c r="B22" s="31" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E22" s="37" t="n">
         <v>1</v>
@@ -3775,13 +3778,13 @@
         <v>15</v>
       </c>
       <c r="B23" s="31" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D23" s="36" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E23" s="37" t="n">
         <v>2</v>
@@ -3808,13 +3811,13 @@
         <v>16</v>
       </c>
       <c r="B24" s="31" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D24" s="36" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E24" s="37" t="n">
         <v>1</v>
@@ -3838,26 +3841,26 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="33" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="14" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H26" s="41" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I26" s="41" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J26" s="41" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="42" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="H27" s="43" t="n">
         <f aca="false">SUMPRODUCT($G$9:$G$24,H$9:H$24)</f>
@@ -3874,7 +3877,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="31" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H28" s="38" t="n">
         <f aca="false">SUMPRODUCT($F$9:$F$24,H$9:H$24)</f>
@@ -3891,7 +3894,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="42" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H29" s="44" t="n">
         <v>280000</v>
@@ -3905,7 +3908,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="31" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H30" s="38" t="n">
         <f aca="false">(H29)*(1+$C$7)</f>
@@ -3922,7 +3925,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="42" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H31" s="43" t="n">
         <f aca="false">(H27)-(H29)</f>
@@ -3939,7 +3942,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="31" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H32" s="45" t="n">
         <f aca="false">IFERROR(1-(H29)/(H27),0)</f>
@@ -3956,7 +3959,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="42" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H33" s="43" t="n">
         <f aca="false">(H29)-(H28)</f>
@@ -3973,7 +3976,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="31" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H34" s="45" t="n">
         <f aca="false">IFERROR(((H29)-(H28))/(H29),0)</f>
@@ -3990,27 +3993,27 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="33" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="22"/>
       <c r="B38" s="22" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C38" s="22"/>
       <c r="D38" s="22" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E38" s="22"/>
       <c r="F38" s="22"/>
       <c r="G38" s="22" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H38" s="22"/>
       <c r="I38" s="22"/>
@@ -4018,26 +4021,26 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="31" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C39" s="31"/>
       <c r="D39" s="46" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E39" s="46"/>
       <c r="F39" s="46"/>
       <c r="G39" s="37" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="H39" s="37"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="31" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C40" s="31"/>
       <c r="D40" s="46" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E40" s="46"/>
       <c r="F40" s="46"/>
@@ -4048,11 +4051,11 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="31" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C41" s="31"/>
       <c r="D41" s="46" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E41" s="46"/>
       <c r="F41" s="46"/>
@@ -4063,11 +4066,11 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="31" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C42" s="31"/>
       <c r="D42" s="46" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E42" s="46"/>
       <c r="F42" s="46"/>
@@ -4078,11 +4081,11 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="31" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C43" s="31"/>
       <c r="D43" s="46" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E43" s="46"/>
       <c r="F43" s="46"/>
@@ -4093,11 +4096,11 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="31" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C44" s="31"/>
       <c r="D44" s="46" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E44" s="46"/>
       <c r="F44" s="46"/>
@@ -4108,11 +4111,11 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="31" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C45" s="31"/>
       <c r="D45" s="46" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E45" s="46"/>
       <c r="F45" s="46"/>
@@ -4123,16 +4126,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="31" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C46" s="31"/>
       <c r="D46" s="46" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E46" s="46"/>
       <c r="F46" s="46"/>
       <c r="G46" s="37" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="H46" s="37"/>
     </row>
@@ -4192,7 +4195,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="47" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C2" s="47"/>
       <c r="D2" s="47"/>
@@ -4201,7 +4204,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -4210,7 +4213,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="48" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C5" s="48"/>
       <c r="D5" s="48"/>
@@ -4219,7 +4222,7 @@
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="49" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C6" s="49"/>
       <c r="D6" s="49"/>
@@ -4228,7 +4231,7 @@
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="49" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C7" s="49"/>
       <c r="D7" s="49"/>
@@ -4237,7 +4240,7 @@
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="49" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C8" s="49"/>
       <c r="D8" s="49"/>
@@ -4246,7 +4249,7 @@
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="48" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C10" s="48"/>
       <c r="D10" s="48"/>
@@ -4255,7 +4258,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="13" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
@@ -4264,7 +4267,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="13" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
@@ -4273,7 +4276,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="13" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
@@ -4282,7 +4285,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="13" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
@@ -4291,7 +4294,7 @@
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="48" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C16" s="48"/>
       <c r="D16" s="48"/>
@@ -4301,18 +4304,18 @@
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C17" s="50"/>
       <c r="D17" s="51" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E17" s="51" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F17" s="51" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C18" s="7" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D18" s="52" t="n">
         <f aca="false">ABONO!H27</f>
@@ -4329,7 +4332,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C19" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D19" s="53" t="n">
         <f aca="false">ABONO!H29</f>
@@ -4346,7 +4349,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C20" s="7" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D20" s="52" t="n">
         <f aca="false">ABONO!H31</f>
@@ -4363,7 +4366,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C21" s="7" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D21" s="54" t="n">
         <f aca="false">ABONO!H32</f>
@@ -4380,7 +4383,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C23" s="55" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D23" s="55"/>
       <c r="E23" s="55"/>
@@ -4388,7 +4391,7 @@
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="48" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C25" s="48"/>
       <c r="D25" s="48"/>
@@ -4397,7 +4400,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="13" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
@@ -4406,7 +4409,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="13" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
@@ -4415,7 +4418,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="13" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
@@ -4424,7 +4427,7 @@
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="48" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C30" s="48"/>
       <c r="D30" s="48"/>
@@ -4433,7 +4436,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="13" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
@@ -4449,7 +4452,7 @@
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="48" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C34" s="48"/>
       <c r="D34" s="48"/>
@@ -4458,7 +4461,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="56" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C35" s="56"/>
       <c r="D35" s="56"/>
@@ -4467,7 +4470,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="56" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C36" s="56"/>
       <c r="D36" s="56"/>
@@ -4476,7 +4479,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="56" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C37" s="56"/>
       <c r="D37" s="56"/>
@@ -4485,7 +4488,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="57" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C39" s="57"/>
       <c r="D39" s="57"/>
@@ -4547,7 +4550,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -4556,19 +4559,19 @@
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4576,13 +4579,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C3" s="36" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="58"/>
     </row>
@@ -4591,13 +4594,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C4" s="36" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E4" s="58"/>
     </row>
@@ -4606,13 +4609,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D5" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E5" s="58"/>
     </row>
@@ -4621,13 +4624,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C6" s="36" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E6" s="58"/>
     </row>
@@ -4636,13 +4639,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C7" s="36" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E7" s="58"/>
     </row>
@@ -4651,13 +4654,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E8" s="58"/>
     </row>
@@ -4666,13 +4669,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C9" s="36" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D9" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E9" s="58"/>
     </row>
@@ -4681,13 +4684,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C10" s="36" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D10" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E10" s="58"/>
     </row>
@@ -4696,13 +4699,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C11" s="36" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E11" s="58"/>
     </row>
@@ -4711,13 +4714,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="24" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D12" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E12" s="58"/>
     </row>
@@ -4726,13 +4729,13 @@
         <v>11</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E13" s="58"/>
     </row>
@@ -4741,13 +4744,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C14" s="36" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D14" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E14" s="58"/>
     </row>
@@ -4756,13 +4759,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E15" s="58"/>
     </row>
@@ -4771,13 +4774,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C16" s="36" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D16" s="31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E16" s="58"/>
     </row>
@@ -4811,48 +4814,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Marcar condición fiscal como a verificar (base ubica a Matheu en zona monotributo)
- Ficha del Excel: condición IVA pendiente de confirmar con constancia
- Informe: hallazgo del barrido de Drive (sin PDF del cliente en Drive,
  fila en bloque monotributo de la base) y primer paso del diagnóstico

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PCAGEfq7p7jhfQiJzYkBZA
</commit_message>
<xml_diff>
--- a/Estudio Contable/CLIENTES/ACT RESP. INSC/MATHEU MARCO/Analisis Integral y Abono - MATHEU MARCO.xlsx
+++ b/Estudio Contable/CLIENTES/ACT RESP. INSC/MATHEU MARCO/Analisis Integral y Abono - MATHEU MARCO.xlsx
@@ -58,7 +58,7 @@
     <t xml:space="preserve">Condición fiscal</t>
   </si>
   <si>
-    <t xml:space="preserve">Responsable Inscripto (según carpeta del estudio)</t>
+    <t xml:space="preserve">A CONFIRMAR: carpeta dice Resp. Inscripto, pero la base lo ubica en zona Monotributo — bajar constancia de inscripción</t>
   </si>
   <si>
     <t xml:space="preserve">Ingresos Brutos</t>
@@ -1953,11 +1953,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>